<commit_message>
23rd commit: Updated unittest plan for SavingsAccount class. Created unit tests for SavingsAccount class and updated all docstrings in savings_account module.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_savings_account.xlsx
+++ b/tests/A02_pixell_test_plan_savings_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>#VALUE!</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Developer:</t>
   </si>
   <si>
-    <t>Student Name</t>
+    <t>Sven Beitenger</t>
   </si>
   <si>
     <t>Class Name:</t>
@@ -58,25 +58,62 @@
     <t>Attributes are set to parameter values.</t>
   </si>
   <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>1172010, 98765, 50000.85, date(2025,9,30), 1000</t>
+  </si>
+  <si>
+    <t>all attributes are set</t>
+  </si>
+  <si>
     <t>minimum_balance has invalid type.</t>
   </si>
   <si>
+    <t>1172010, 98765, 50000.85, date(2025,9,30), "str"</t>
+  </si>
+  <si>
+    <t>minimum_balance = 50</t>
+  </si>
+  <si>
     <t>get_service_charges</t>
   </si>
   <si>
     <t>balance greater than minimum balance</t>
   </si>
   <si>
+    <t>SavingsAccount(1172010, 98765, 50000.85, date(2025,9,30), 1000)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>service_charge = 0.50</t>
+  </si>
+  <si>
     <t>balance  equal to minimum balance</t>
   </si>
   <si>
+    <t>1172010, 98765, 1000, date(2025,9,30), 1000</t>
+  </si>
+  <si>
     <t>balance less than minimum balance</t>
   </si>
   <si>
+    <t>1172010, 98765, 500, date(2025,9,30), 1000</t>
+  </si>
+  <si>
+    <t>serivce_charge = 1.00</t>
+  </si>
+  <si>
     <t>__str__</t>
   </si>
   <si>
     <t>appropriate value returned based on attribute values.</t>
+  </si>
+  <si>
+    <t>Account Number: 1172010 Balance: 50,000.85
+Minimum Balance: 1,000.00 Account Type: Savings</t>
   </si>
   <si>
     <t>Add more rows as necessary</t>
@@ -911,7 +948,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="16">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="55.5" customFormat="1" s="16">
       <c r="A7" s="17"/>
       <c r="B7" s="18">
         <v>1</v>
@@ -922,11 +959,17 @@
       <c r="D7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="16">
+      <c r="E7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="78.75" customFormat="1" s="16">
       <c r="A8" s="17"/>
       <c r="B8" s="21">
         <v>2</v>
@@ -935,71 +978,101 @@
         <v>12</v>
       </c>
       <c r="D8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="31.5" customFormat="1" s="16">
+      <c r="F8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="64.5" customFormat="1" s="16">
       <c r="A9" s="17"/>
       <c r="B9" s="18">
         <v>3</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5" customFormat="1" s="16">
+        <v>21</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="57" customFormat="1" s="16">
       <c r="A10" s="17"/>
       <c r="B10" s="18">
         <v>4</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5" customFormat="1" s="16">
+        <v>25</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="69" customFormat="1" s="16">
       <c r="A11" s="17"/>
       <c r="B11" s="21">
         <v>5</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="31.5" customFormat="1" s="16">
+        <v>27</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="77.25" customFormat="1" s="16">
       <c r="A12" s="17"/>
       <c r="B12" s="18">
         <v>6</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
+        <v>31</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1"/>
@@ -1233,7 +1306,7 @@
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="1"/>
       <c r="B34" s="26" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>

</xml_diff>